<commit_message>
Update training roster and preference files
Update three spreadsheet files: MASTER Education Classes Roster, Preferences v6, and Requirements with current data.  Noland changed to Seyoum, Dinardo removed
</commit_message>
<xml_diff>
--- a/upload files/Requirements.xlsx
+++ b/upload files/Requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaronbell/Desktop/Git Repo Clone/CrewOps360/upload files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04C659C-86EB-8445-BD14-98CBB236BDF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9F3E5FC-27DD-0048-9BCA-8A3BB1C5D369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17260" xr2:uid="{10D55376-794F-6145-963B-6A2FF77FD7A3}"/>
   </bookViews>
@@ -176,9 +176,6 @@
     <t>McGrath</t>
   </si>
   <si>
-    <t>Noland</t>
-  </si>
-  <si>
     <t>Murphy</t>
   </si>
   <si>
@@ -330,6 +327,9 @@
   </si>
   <si>
     <t>Michael.Pepin@bostonmedflight.org</t>
+  </si>
+  <si>
+    <t>Seyoum</t>
   </si>
 </sst>
 </file>
@@ -876,7 +876,7 @@
         <v>5</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -904,7 +904,7 @@
         <v>5</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -932,7 +932,7 @@
         <v>5</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -949,7 +949,7 @@
         <v>2</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -983,7 +983,7 @@
         <v>5</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -1022,7 +1022,7 @@
         <v>5</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -1039,7 +1039,7 @@
         <v>3</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -1056,7 +1056,7 @@
         <v>5</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -1073,7 +1073,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -1282,7 +1282,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>46</v>
+        <v>97</v>
       </c>
       <c r="B40" s="2">
         <v>3</v>
@@ -1296,7 +1296,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B41" s="1">
         <v>6</v>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>7</v>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B43" s="1">
         <v>6</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B44" s="1">
         <v>6</v>
@@ -1349,7 +1349,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B45" s="1">
         <v>6</v>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B46" s="1">
         <v>6</v>
@@ -1377,7 +1377,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B47" s="1">
         <v>6</v>
@@ -1391,7 +1391,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B48" s="1">
         <v>6</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B49" s="1">
         <v>6</v>
@@ -1419,7 +1419,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B50" s="1">
         <v>6</v>
@@ -1433,7 +1433,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B51" s="1">
         <v>6</v>
@@ -1447,7 +1447,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B52" s="1">
         <v>6</v>
@@ -1461,7 +1461,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B53" s="1">
         <v>6</v>
@@ -1475,7 +1475,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B54" s="1">
         <v>6</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B55" s="1">
         <v>6</v>
@@ -1503,7 +1503,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B56" s="1">
         <v>6</v>
@@ -1517,7 +1517,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B57" s="1">
         <v>6</v>
@@ -1531,7 +1531,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B58" s="1">
         <v>6</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B59" s="1">
         <v>6</v>
@@ -1559,7 +1559,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B60" s="1">
         <v>6</v>
@@ -1573,7 +1573,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B61" s="1">
         <v>6</v>
@@ -1587,7 +1587,7 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B62" s="1">
         <v>6</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B63" s="1">
         <v>6</v>
@@ -1615,7 +1615,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B64" s="1">
         <v>6</v>
@@ -1629,7 +1629,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B65" s="1">
         <v>6</v>
@@ -1643,7 +1643,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B66" s="1">
         <v>6</v>
@@ -1657,7 +1657,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>7</v>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B68" s="1">
         <v>6</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B69" s="1">
         <v>6</v>
@@ -1696,7 +1696,7 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B70" s="1">
         <v>6</v>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B71" s="1">
         <v>6</v>
@@ -1724,7 +1724,7 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B72" s="1">
         <v>6</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B73" s="1">
         <v>6</v>
@@ -1752,7 +1752,7 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B74" s="1">
         <v>6</v>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B75" s="1">
         <v>6</v>
@@ -1780,7 +1780,7 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B76" s="1">
         <v>6</v>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B77" s="1">
         <v>6</v>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B78" s="1">
         <v>6</v>
@@ -1822,7 +1822,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B79" s="1">
         <v>6</v>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B80" s="1">
         <v>6</v>
@@ -1850,7 +1850,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B81" s="1">
         <v>6</v>
@@ -1864,7 +1864,7 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B82" s="1">
         <v>6</v>
@@ -2065,20 +2065,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2101,14 +2101,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FC3EAF2-EF9F-4ED7-9C58-0B29683A52D2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E8E94FF-6E53-4E14-A123-F68683276D30}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2116,4 +2108,12 @@
     <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FC3EAF2-EF9F-4ED7-9C58-0B29683A52D2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>